<commit_message>
add: adição da revisão e do historico de prompts
</commit_message>
<xml_diff>
--- a/HistóricoDoMeuExperimento.xlsx
+++ b/HistóricoDoMeuExperimento.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="110">
   <si>
     <t>Prompt</t>
   </si>
@@ -64,25 +64,55 @@
 create too the skills.md and explain that</t>
   </si>
   <si>
+    <t>Bom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usaria novamente o prompt </t>
+  </si>
+  <si>
+    <t>Fez um bom planejamento e uma boa base para iniciar a implementação do sistema</t>
+  </si>
+  <si>
     <t>haja como um gerente especialista em banco de dados e adicione com as melhores instruções no skill e no project-config as configurações necessárias para ter um banco mongoDB</t>
   </si>
   <si>
+    <t>Muito bom</t>
+  </si>
+  <si>
     <t>alterou corretamente os arquivos pedidos</t>
   </si>
   <si>
     <t>Agora haja como um senior fullstack, especialista em desenvolvimento de código na linguagem ts e em configuração com o mongoDB e construa o sistema seguindo cada passo dos arquivos selecionados (skill.md e project-config.yaml)</t>
   </si>
   <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>Acho que detalhando mais, iria ser melhor</t>
+  </si>
+  <si>
     <t>Criou uma boa estrutura básica, entretando alguns arquivos .md que achei desnecessários e o sistema dá erro ao build</t>
   </si>
   <si>
     <t>faça o build e rode o sistema, corriga os erros, deixe os códigos mais légiveis e implemente mais funcionalidades no frontend que ainda não foram desenvolvidas</t>
   </si>
   <si>
+    <t>ruim</t>
+  </si>
+  <si>
+    <t>Não gostei do resultado</t>
+  </si>
+  <si>
     <t>acabou demorando muito tempo para testar o build e se perdeu, tive que pular essa etapa. Fez algumas alterações no código, mas não executou bem, tive que pedir para testar o build novamente, dessa vez de forma isolada no prompt seguinte</t>
   </si>
   <si>
     <t>faça o build e rode o sistema, corriga os erros que tão interferindo na build do sistema</t>
+  </si>
+  <si>
+    <t>bom</t>
+  </si>
+  <si>
+    <t>gostei do resultado</t>
   </si>
   <si>
     <t>Agora corrigiu os erros de build</t>
@@ -171,6 +201,9 @@
 CSV com o gabarito de cada prova. Cada linha do CSV contém informações sobre uma
 prova: o número da prova, seguido do gabarito de cada questão da prova (as letras que
 deveriam ser selecionadas, ou o somatório esperado).</t>
+  </si>
+  <si>
+    <t>não gostei do resultado</t>
   </si>
   <si>
     <t>Não desenvolveu corretamente, gerou um pdf à partir da prova, entretanto não foi com o formato certo que foi pedido</t>
@@ -768,13 +801,13 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="4" width="37.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="13.005" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="4" width="15.147857142857141" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="4" width="18.433571428571426" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="4" width="37.57642857142857" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -798,541 +831,731 @@
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="378">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="366">
       <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
+      <c r="C3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
       <c r="A4" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
+      <c r="C4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E4" s="2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
       <c r="A5" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="E5" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
+      <c r="C6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="E6" s="2" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
       <c r="A7" s="2" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
+      <c r="C7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="E7" s="2" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18">
       <c r="A8" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
+      <c r="C8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="E8" s="2" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
       <c r="A9" s="2" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
+      <c r="C9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E9" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18">
+      <c r="A10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18">
+      <c r="A11" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18">
+      <c r="A12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18">
+      <c r="A13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18">
+      <c r="A14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="22.5">
-      <c r="A10" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="22.5">
-      <c r="A11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="22.5">
-      <c r="A12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="22.5">
-      <c r="A13" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="22.5">
-      <c r="A14" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
       <c r="E14" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="22.5">
+        <v>37</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="30">
       <c r="A15" s="2" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
+      <c r="C15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="E15" s="2" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="22.5">
       <c r="A16" s="2" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
+      <c r="C16" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="E16" s="2" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="22.5">
       <c r="A17" s="2" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
+      <c r="C17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="E17" s="2" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="22.5">
       <c r="A18" s="2" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
+      <c r="C18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="E18" s="2" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="22.5">
       <c r="A19" s="2" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
+      <c r="C19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="E19" s="2" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="22.5">
       <c r="A20" s="2" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
+      <c r="C20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="E20" s="2" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="22.5">
       <c r="A21" s="2" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
+      <c r="C21" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E21" s="2" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="22.5">
       <c r="A22" s="2" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
+      <c r="C22" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E22" s="2" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="22.5">
       <c r="A23" s="2" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
+      <c r="C23" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E23" s="2" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="22.5">
       <c r="A24" s="2" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="22.5">
       <c r="A25" s="2" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
+      <c r="C25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="E25" s="2" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="22.5">
       <c r="A26" s="2" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
+      <c r="C26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="E26" s="2" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="22.5">
       <c r="A27" s="2" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
+      <c r="C27" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="E27" s="2" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="22.5">
       <c r="A28" s="2" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
+      <c r="C28" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="E28" s="2" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="22.5">
       <c r="A29" s="2" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
+      <c r="C29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E29" s="2" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="22.5">
       <c r="A30" s="2" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
+      <c r="C30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="E30" s="2" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="22.5">
       <c r="A31" s="2" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
+      <c r="C31" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="E31" s="2" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="22.5">
       <c r="A32" s="2" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
+      <c r="C32" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="E32" s="2" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="22.5">
       <c r="A33" s="2" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
+      <c r="C33" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="E33" s="2" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="22.5">
       <c r="A34" s="2" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
+      <c r="C34" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E34" s="2" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="22.5">
       <c r="A35" s="2" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
+      <c r="C35" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="E35" s="2" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="22.5">
       <c r="A36" s="2" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
+      <c r="C36" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="E36" s="2" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="22.5">
       <c r="A37" s="2" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
+      <c r="C37" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E37" s="2" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="22.5">
       <c r="A38" s="2" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
+      <c r="C38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="E38" s="2" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="22.5">
       <c r="A39" s="2" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
+      <c r="C39" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="E39" s="2" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="22.5">
       <c r="A40" s="2" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
+      <c r="C40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="E40" s="2" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="22.5">
       <c r="A41" s="2" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
+      <c r="C41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="E41" s="2" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="22.5">
       <c r="A42" s="2" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
+      <c r="C42" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="E42" s="2" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="22.5">
       <c r="A43" s="2" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="2" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="22.5">
       <c r="A44" s="2" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
+      <c r="C44" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E44" s="2" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="22.5">
       <c r="A45" s="2" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
+      <c r="C45" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E45" s="2" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="22.5">
       <c r="A46" s="2" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
+      <c r="C46" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E46" s="2" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="22.5">
       <c r="A47" s="2" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
+      <c r="C47" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E47" s="2" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="22.5">
       <c r="A48" s="2" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
+      <c r="C48" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="E48" s="2" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="22.5">
       <c r="A49" s="2" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="B49" s="2"/>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
+      <c r="C49" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E49" s="2" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="22.5">
       <c r="A50" s="2" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="B50" s="2"/>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
+      <c r="C50" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E50" s="2" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="22.5">
       <c r="A51" s="2" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
+      <c r="C51" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="E51" s="2" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="22.5">

</xml_diff>